<commit_message>
fix: clarify q1 v3 success aliases
</commit_message>
<xml_diff>
--- a/第一问_30天路线优化材料包/09_Q1_V3_鲁棒联合优化/reports/新疆旅游第一问Q1_V3鲁棒联合优化结果.xlsx
+++ b/第一问_30天路线优化材料包/09_Q1_V3_鲁棒联合优化/reports/新疆旅游第一问Q1_V3鲁棒联合优化结果.xlsx
@@ -2597,7 +2597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2893,6 +2893,43 @@
       <c r="G8" t="inlineStr">
         <is>
           <t>安装OR-Tools/Gurobi后构建小规模MILP/CP-SAT定向游精确模型</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>V3-A8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>success_metrics</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>success_probability为历史兼容字段，等同于operational_success_probability</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>implemented_alias</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>outputs/q1_v3_simulation_summary.csv</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>旧代码可能继续读取success_probability，需要在论文和报告中优先展示拆分后的两类成功率</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>下一个大版本可移除兼容字段或重命名为operational_success_probability</t>
         </is>
       </c>
     </row>

</xml_diff>